<commit_message>
Close two gaps found in the final pass
The flag border was a literal with an override on [data-theme="dark"].
That attribute is absent in the default "system" setting, which is what
most readers are on, so a reader whose OS is dark got a near-black edge
on a near-black ground. It is a token now, defined in all three theme
states like every other colour, and an audit of the built stylesheet
confirms all fifteen tokens are.

The workbook did not know about the locations the dashboard reports.
Two deliverables of one study disagreed about what it covers, and the
workbook is the one that gets forwarded, so it now carries the ten
priced-but-unranked locations and the three reasons a location can be
absent. The year column also needed a format; without one Excel renders
2025 as 2,025.
</commit_message>
<xml_diff>
--- a/gbs-location-selection.xlsx
+++ b/gbs-location-selection.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Criteria &amp; weights" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="City ranking" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Wage gap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Not ranked" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <name val="Calibri"/>
@@ -104,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +153,18 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
@@ -3522,4 +3537,388 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GBS &amp; GCC LOCATION SELECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Locations outside the ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Five pillars reach these markets because ILOSTAT and the World Bank cover every country alike. Capability and employer depth do not, and those are the two the job postings carry, so nothing here is scored or ranked against the cities that are.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Cost USD / month</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Observed</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Relevant workforce</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Hours shared with HQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Prague</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>3127.649739729742</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>2352383</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>75.02690106</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Bucharest</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Romania</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>2205.205546047026</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>2346761</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>60.14429548</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>San José</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Costa Rica</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>1658.844198230243</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>722616</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>67.2234613</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Lisbon</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>1622.446997552137</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>2205427</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>70.26399764</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>1452.993599350319</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>2170460</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>60.70442944</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>904.4593513387189</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>5647196</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>65.60742774000001</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>716.7530708855829</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>5959091</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>48.56104388</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Santo Domingo</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>645.8720670166648</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>1272228</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>56.63891526</v>
+      </c>
+      <c r="G13" s="22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Manila</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>505.3461322199106</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>9208417</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>49.2408423</v>
+      </c>
+      <c r="G14" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>478.1951984488104</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>7277217</v>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>52.10275567999999</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Three other kinds of absence</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Seen but too thin: 105 locations appear in the sample and clear neither threshold. Closest are Gdańsk (7 postings, 3 employers), Katowice (7 postings, 3 employers), Delhi (6 postings, 3 employers), Łódź (4 postings, 3 employers). The employer count is usually what stops them, and one employer hiring is an office rather than a centre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Not priceable: China (Wuxi, Dalian, Chengdu) and Morocco (Casablanca, Rabat). ILOSTAT publishes no earnings by occupation for either, so there is no cost figure on the basis every market here uses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Incoherent: Egypt reports professionals at 1.06x clerical pay against 1.3-2.9x in every other market, so it is excluded by test rather than by judgement.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A18:G18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Let the notes use the measure, and cut what they did not need
The footnotes were capped at 70ch and the source line at 92ch, so both
stopped around half way across while the table beside them used the full
width. Dropping the cap alone would have given a 105-character line, so
they run in two columns instead: the width is filled and the line stays
readable. Print keeps one column, where the measure is already narrow and
the page count is decided by a few points.

Three things left the exhibit. The near-miss list ran to six locations
with two figures each, which is a list rather than a finding; three carry
it. The argument that a second job board would not close the coverage gap
answers an objection instead of helping anyone read the table, so it moved
to the method section where the other objections live. And one column
mixed units -- 722,616 beside 2.4m made the reader do the conversion.
</commit_message>
<xml_diff>
--- a/gbs-location-selection.xlsx
+++ b/gbs-location-selection.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -653,26 +653,33 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>•  Exhibit 3 subtracts a national baseline from cities that sometimes carry a regional index, so a capital-city premium sits on one side of it and not the other. Warsaw against a UK baseline is the clearest case: it reads as dearer than the UK, which is partly Mazowieckie against a British national mean rather than a wage fact.</t>
+          <t>•  A second job board would not close the coverage gap. Employer depth counts distinct employers within one feed, so another feed’s count is not comparable, and splicing one in would move Manila into the ranking on evidence unlike the rest.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>•  Exhibit 3 is a wage line, not a business case. It excludes facilities, technology, management overhead, transition and severance, and holds headcount one-for-one. Read it as the upper bound on one component of the saving.</t>
+          <t>•  Exhibit 3 subtracts a national baseline from cities that sometimes carry a regional index, so a capital-city premium sits on one side of it and not the other. Warsaw against a UK baseline is the clearest case: it reads as dearer than the UK, which is partly Mazowieckie against a British national mean rather than a wage fact.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>•  Exhibit 3 is a wage line, not a business case. It excludes facilities, technology, management overhead, transition and severance, and holds headcount one-for-one. Read it as the upper bound on one component of the saving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>•  Six established locations sit outside the ranking because the postings feed does not reach them: Manila, Kuala Lumpur, Bucharest, Prague, Budapest and Lisbon. Five pillars do reach them and are reported under 'Beyond the sample'; capability and employer depth are the two that cannot be, so these markets are never scored against the ranked cities.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Postings sample: August 2026.  Method and code: github.com/morichtereur/gbs-location-selection</t>
         </is>

</xml_diff>

<commit_message>
Close on the checks a phase 2 would actually run
The page ends on what would change it: live wage and employer-charge
quotes for the top band, whose cost is mostly a national figure under a
uniform loading assumption; site visits against a capability pillar that
rests on as few as four postings per city; and attrition and ramp data
from the employers already operating there, since the backfill uplift is
the one Exhibit 3 input that can reorder cities and today it is a
slider. Framed as what this analysis cannot settle, written from the run
on screen, and mirrored in the pre-script document. The dashboard and
workbook artifacts are rebuilt here for the tree as a whole.
</commit_message>
<xml_diff>
--- a/gbs-location-selection.xlsx
+++ b/gbs-location-selection.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -646,42 +646,35 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>•  One snapshot. A city hiring quietly during the fetch is under-represented; absence is weak evidence, not a verdict.</t>
+          <t>•  A second job board would not close the coverage gap. Employer depth counts distinct employers within one feed, so another feed’s count is not comparable, and splicing one in would move Manila into the ranking on evidence unlike the rest.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>•  A second job board would not close the coverage gap. Employer depth counts distinct employers within one feed, so another feed’s count is not comparable, and splicing one in would move Manila into the ranking on evidence unlike the rest.</t>
+          <t>•  Exhibit 3 subtracts a national baseline from cities that sometimes carry a regional index, so a capital-city premium sits on one side of it and not the other. Warsaw against a UK baseline is the clearest case: it reads as dearer than the UK, which is partly Mazowieckie against a British national mean rather than a wage fact.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>•  Exhibit 3 subtracts a national baseline from cities that sometimes carry a regional index, so a capital-city premium sits on one side of it and not the other. Warsaw against a UK baseline is the clearest case: it reads as dearer than the UK, which is partly Mazowieckie against a British national mean rather than a wage fact.</t>
+          <t>•  Exhibit 3 is a wage line, not a business case. It excludes facilities, technology, management overhead, transition and severance, and holds headcount one-for-one. Read it as the upper bound on one component of the saving.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>•  Exhibit 3 is a wage line, not a business case. It excludes facilities, technology, management overhead, transition and severance, and holds headcount one-for-one. Read it as the upper bound on one component of the saving.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
           <t>•  Six established locations sit outside the ranking because the postings feed does not reach them: Manila, Kuala Lumpur, Bucharest, Prague, Budapest and Lisbon. Five pillars do reach them and are reported under 'Beyond the sample'; capability and employer depth are the two that cannot be, so these markets are never scored against the ranked cities.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Postings sample: August 2026.  Method and code: github.com/morichtereur/gbs-location-selection</t>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Postings sample: 22 August 2026.  Method and code: github.com/morichtereur/gbs-location-selection</t>
         </is>
       </c>
     </row>
@@ -787,11 +780,7 @@
           <t>ILOSTAT earnings by occupation</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>2020–2025</t>
-        </is>
-      </c>
+      <c r="E6" s="9" t="n"/>
       <c r="F6" s="10" t="n">
         <v>0.3</v>
       </c>
@@ -820,11 +809,7 @@
           <t>ILOSTAT employment by occupation</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
+      <c r="E7" s="11" t="n"/>
       <c r="F7" s="12" t="n">
         <v>0.18</v>
       </c>
@@ -853,11 +838,7 @@
           <t>World Bank Worldwide Governance Indicators</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
+      <c r="E8" s="9" t="n"/>
       <c r="F8" s="10" t="n">
         <v>0.09</v>
       </c>
@@ -886,11 +867,7 @@
           <t>Adzuna job postings</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>Aug 2026</t>
-        </is>
-      </c>
+      <c r="E9" s="11" t="n"/>
       <c r="F9" s="12" t="n">
         <v>0.13</v>
       </c>
@@ -952,11 +929,7 @@
           <t>ILOSTAT, derived</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>2015–2025</t>
-        </is>
-      </c>
+      <c r="E11" s="11" t="n"/>
       <c r="F11" s="12" t="n">
         <v>0.09</v>
       </c>
@@ -985,11 +958,7 @@
           <t>Adzuna job postings</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Aug 2026</t>
-        </is>
-      </c>
+      <c r="E12" s="9" t="n"/>
       <c r="F12" s="10" t="n">
         <v>0.12</v>
       </c>
@@ -2368,14 +2337,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:S58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -3521,21 +3490,314 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>A positive figure is the annual wage the move takes out per role; a negative one means the city is dearer than the origin.</t>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Fully loaded, against the default origin</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>The origin is always a national figure while the Polish cities carry a regional index, so a capital-city premium sits on one side of the subtraction and not the other.</t>
+          <t>Employer loading 25% of gross wage, applied to origin and destination alike. Attrition backfill 15%, applied to the destination only, since the origin is not being stood up. Projection horizon 0 years, at each market's own measured wage drift.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>The first two are assumptions, not measurements. No free source gives comparable employer-charge schedules for all eleven markets, so the factor is uniform — which scales every gap and cannot reorder them. Real charges differ sharply by country, and pricing that difference is exactly what this study cannot do. Change the numbers in src/config.py to re-run on your own. Origin: Switzerland.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Loaded cost USD / month</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Base gap vs Switzerland</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Loaded gap vs Switzerland</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>City-level wage?</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Warsaw</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="n">
+        <v>6789.216886855975</v>
+      </c>
+      <c r="C42" s="16" t="n">
+        <v>42744.17687174902</v>
+      </c>
+      <c r="D42" s="16" t="n">
+        <v>42803.62074504215</v>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>Kraków</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="n">
+        <v>5478.102168209887</v>
+      </c>
+      <c r="C43" s="18" t="n">
+        <v>53689.13452305548</v>
+      </c>
+      <c r="D43" s="18" t="n">
+        <v>58536.9973687952</v>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Wrocław</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="n">
+        <v>4260.923559942105</v>
+      </c>
+      <c r="C44" s="16" t="n">
+        <v>63849.92986163872</v>
+      </c>
+      <c r="D44" s="16" t="n">
+        <v>73143.14066800858</v>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Poznań</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="n">
+        <v>3261.88371955932</v>
+      </c>
+      <c r="C45" s="18" t="n">
+        <v>72189.74070309501</v>
+      </c>
+      <c r="D45" s="18" t="n">
+        <v>85131.61875260199</v>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="n">
+        <v>1227.73778350239</v>
+      </c>
+      <c r="C46" s="16" t="n">
+        <v>89170.43721278764</v>
+      </c>
+      <c r="D46" s="16" t="n">
+        <v>109541.3699852852</v>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="n">
+        <v>1202.385660718941</v>
+      </c>
+      <c r="C47" s="18" t="n">
+        <v>89382.07232471905</v>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>109845.5954586866</v>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="B48" s="16" t="n">
+        <v>491.6612147170598</v>
+      </c>
+      <c r="C48" s="16" t="n">
+        <v>95315.07639569127</v>
+      </c>
+      <c r="D48" s="16" t="n">
+        <v>118374.2888107091</v>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="n">
+        <v>491.6612147170598</v>
+      </c>
+      <c r="C49" s="18" t="n">
+        <v>95315.07639569127</v>
+      </c>
+      <c r="D49" s="18" t="n">
+        <v>118374.2888107091</v>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>491.6612147170598</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <v>95315.07639569127</v>
+      </c>
+      <c r="D50" s="16" t="n">
+        <v>118374.2888107091</v>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="n">
+        <v>491.6612147170598</v>
+      </c>
+      <c r="C51" s="18" t="n">
+        <v>95315.07639569127</v>
+      </c>
+      <c r="D51" s="18" t="n">
+        <v>118374.2888107091</v>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="B52" s="16" t="n">
+        <v>491.6612147170598</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <v>95315.07639569127</v>
+      </c>
+      <c r="D52" s="16" t="n">
+        <v>118374.2888107091</v>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>national wage</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>A positive figure is the annual wage the move takes out per role; a negative one means the city is dearer than the origin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>The grid above is the gross wage line. The loaded figures are in the block beneath it, and are not a fixed multiple of the grid: the attrition uplift applies to the destination only, so it moves cheap and dear cities by different amounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>The origin is always a national figure while the Polish cities carry a regional index, so a capital-city premium sits on one side of the subtraction and not the other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>A city marked 'national wage' has no city-level earnings in any reachable source, so neither side of its gap carries a city premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>Germany's earnings come from EU-SILC where the others come from labour force surveys, and Germany (2022) and Singapore (2021) are the oldest observations in the set.</t>
         </is>

</xml_diff>